<commit_message>
Accept system agent export in FA tool and restrict FA to LP title
Agent sheet is now read by header name, so the HR system export can be
pasted as-is. Adds Title/AgentStatus to tblAgent (auto-migrated for
existing data files) and excludes non-LP titles from FA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bj7Lc5F4BSWTnmkMiHmzyc
</commit_message>
<xml_diff>
--- a/tools/access-fa/FA_Input_Mau.xlsx
+++ b/tools/access-fa/FA_Input_Mau.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -493,93 +493,114 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Title: chức danh (LP, PM, PD...). FA chỉ tính cho LP</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sheet Holiday – ngày lễ rơi vào ngày làm việc (để tính số ngày làm việc của tháng)</t>
+          <t xml:space="preserve">  Có thể dán thẳng file xuất hệ thống vào sheet Agent: tool tự nhận cột AGENT_CODE, FULL_NAME, APPOINTMENT_DATE,</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AGENCY_TYPE, TERMINATION_DATE, TITLE (Code), AGENT_STATUS (các cột khác bỏ qua)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Sheet FA_Input – số liệu từng LP theo tháng và kỳ chi trả</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Period: tháng tính, dạng YYYYMM (ví dụ 202610)</t>
+          <t>Sheet Holiday – ngày lễ rơi vào ngày làm việc (để tính số ngày làm việc của tháng)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ky: kỳ chi trả 1–4 (mục D.l). Mỗi kỳ nhập số LŨY KẾ đến ngày chốt ACK của kỳ đó</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ActualDays: số ngày đi làm thực tế trong tháng (gồm cả ngày làm thêm theo yêu cầu)</t>
+          <t>Sheet FA_Input – số liệu từng LP theo tháng và kỳ chi trả</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FYC: FYC phát sinh (VND) | Contracts: số hợp đồng phát sinh (cho phép 0,5)</t>
+          <t xml:space="preserve">  Period: tháng tính, dạng YYYYMM (ví dụ 202610)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Recruits: số LP giới thiệu trong tháng</t>
+          <t xml:space="preserve">  Ky: kỳ chi trả 1–4 (mục D.l). Mỗi kỳ nhập số LŨY KẾ đến ngày chốt ACK của kỳ đó</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  K2Pct: %K2 dạng số, ví dụ 85 = 85%. Để TRỐNG nếu chưa có K2 (N/A)</t>
+          <t xml:space="preserve">  ActualDays: số ngày đi làm thực tế trong tháng (gồm cả ngày làm thêm theo yêu cầu)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MDRTPrev: 1 = đạt MDRT năm liền kề trước, 0 = không</t>
+          <t xml:space="preserve">  FYC: FYC phát sinh (VND) | Contracts: số hợp đồng phát sinh (cho phép 0,5)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  TrainingDone: 1 = đã hoàn tất huấn luyện bắt buộc, 0 = chưa</t>
+          <t xml:space="preserve">  Recruits: số LP giới thiệu trong tháng</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  StatusEOM: tình trạng cuối tháng (Active / SE / ...)</t>
+          <t xml:space="preserve">  K2Pct: %K2 dạng số, ví dụ 85 = 85%. Để TRỐNG nếu chưa có K2 (N/A)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MDRTPrev: 1 = đạt MDRT năm liền kề trước, 0 = không</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TrainingDone: 1 = đã hoàn tất huấn luyện bắt buộc, 0 = chưa</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  StatusEOM: tình trạng cuối tháng (Active / SE / ...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Sheet KetQua_KyVong: kết quả tính tay bằng bản đối chiếu Python – dùng để đối soát với tool, tool không đọc sheet này.</t>
         </is>
@@ -596,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -604,6 +625,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -632,6 +654,11 @@
           <t>TerminateDate</t>
         </is>
       </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -652,6 +679,11 @@
           <t>FT</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -672,6 +704,11 @@
           <t>FT</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -692,6 +729,11 @@
           <t>FT</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -712,6 +754,11 @@
           <t>FT</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -732,6 +779,11 @@
           <t>FT</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -752,6 +804,11 @@
           <t>FT</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -772,6 +829,11 @@
           <t>FT</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -792,6 +854,11 @@
           <t>PT</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -812,6 +879,11 @@
           <t>FT</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -830,6 +902,36 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>FT</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PM001</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ngô Thị M</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>46083</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PM</t>
         </is>
       </c>
     </row>
@@ -894,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1362,6 +1464,44 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PM001</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>26000000</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1373,7 +1513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1976,6 +2116,59 @@
       </c>
       <c r="O11" s="6" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PM001</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Chức danh PM → không có FA</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>10500000</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>Chức danh không phải LP (FA chỉ áp dụng LP toàn thời gian)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Use 98-column HR export layout as the standard Agent template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bj7Lc5F4BSWTnmkMiHmzyc
</commit_message>
<xml_diff>
--- a/tools/access-fa/FA_Input_Mau.xlsx
+++ b/tools/access-fa/FA_Input_Mau.xlsx
@@ -71,8 +71,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -474,42 +474,38 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sheet Agent – danh sách LP (nhập 1 lần, cập nhật khi có thay đổi)</t>
+          <t>Sheet Agent – danh sách agent hàng tháng: dán NGUYÊN file xuất hệ thống (Tbl_Agent, 98 cột, giữ đúng tên và thứ tự cột)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AgentCode: mã đại lý | AgentName: họ tên | AppointDate: ngày bổ nhiệm (ngày HĐ đại lý hiệu lực)</t>
+          <t xml:space="preserve">  Cột bắt buộc: Period, AGENT_CODE, FULL_NAME, TITLE (Code), AGENCY_TYPE (FT/PT), APPOINTMENT_DATE</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WorkModel: FT = toàn thời gian, PT = bán thời gian | TerminateDate: ngày chấm dứt HĐ (để trống nếu còn hiệu lực)</t>
+          <t xml:space="preserve">  TERMINATION_DATE để trống nếu HĐ còn hiệu lực. FA chỉ tính cho chức danh LP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Title: chức danh (LP, PM, PD...). FA chỉ tính cho LP</t>
+          <t xml:space="preserve">  Nạp lại cùng Period thì ghi đè đúng tháng đó; các tháng khác giữ nguyên trong lịch sử</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Có thể dán thẳng file xuất hệ thống vào sheet Agent: tool tự nhận cột AGENT_CODE, FULL_NAME, APPOINTMENT_DATE,</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AGENCY_TYPE, TERMINATION_DATE, TITLE (Code), AGENT_STATUS (các cột khác bỏ qua)</t>
+          <t>Sheet Holiday – ngày lễ rơi vào ngày làm việc (để tính số ngày làm việc của tháng)</t>
         </is>
       </c>
     </row>
@@ -519,88 +515,78 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sheet Holiday – ngày lễ rơi vào ngày làm việc (để tính số ngày làm việc của tháng)</t>
+          <t>Sheet FA_Input – số liệu từng LP theo tháng và kỳ chi trả</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Period: tháng tính, dạng YYYYMM (ví dụ 202610)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sheet FA_Input – số liệu từng LP theo tháng và kỳ chi trả</t>
+          <t xml:space="preserve">  Ky: kỳ chi trả 1–4 (mục D.l). Mỗi kỳ nhập số LŨY KẾ đến ngày chốt ACK của kỳ đó</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Period: tháng tính, dạng YYYYMM (ví dụ 202610)</t>
+          <t xml:space="preserve">  ActualDays: số ngày đi làm thực tế trong tháng (gồm cả ngày làm thêm theo yêu cầu)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ky: kỳ chi trả 1–4 (mục D.l). Mỗi kỳ nhập số LŨY KẾ đến ngày chốt ACK của kỳ đó</t>
+          <t xml:space="preserve">  FYC: FYC phát sinh (VND) | Contracts: số hợp đồng phát sinh (cho phép 0,5)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ActualDays: số ngày đi làm thực tế trong tháng (gồm cả ngày làm thêm theo yêu cầu)</t>
+          <t xml:space="preserve">  Recruits: số LP giới thiệu trong tháng</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FYC: FYC phát sinh (VND) | Contracts: số hợp đồng phát sinh (cho phép 0,5)</t>
+          <t xml:space="preserve">  K2Pct: %K2 dạng số, ví dụ 85 = 85%. Để TRỐNG nếu chưa có K2 (N/A)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Recruits: số LP giới thiệu trong tháng</t>
+          <t xml:space="preserve">  MDRTPrev: 1 = đạt MDRT năm liền kề trước, 0 = không</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  K2Pct: %K2 dạng số, ví dụ 85 = 85%. Để TRỐNG nếu chưa có K2 (N/A)</t>
+          <t xml:space="preserve">  TrainingDone: 1 = đã hoàn tất huấn luyện bắt buộc, 0 = chưa</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MDRTPrev: 1 = đạt MDRT năm liền kề trước, 0 = không</t>
+          <t xml:space="preserve">  StatusEOM: tình trạng cuối tháng (Active / SE / ...)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  TrainingDone: 1 = đã hoàn tất huấn luyện bắt buộc, 0 = chưa</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  StatusEOM: tình trạng cuối tháng (Active / SE / ...)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
         <is>
           <t>Sheet KetQua_KyVong: kết quả tính tay bằng bản đối chiếu Python – dùng để đối soát với tool, tool không đọc sheet này.</t>
         </is>
@@ -617,323 +603,1249 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:CT12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="16" customWidth="1" min="35" max="35"/>
+    <col width="16" customWidth="1" min="36" max="36"/>
+    <col width="16" customWidth="1" min="37" max="37"/>
+    <col width="16" customWidth="1" min="38" max="38"/>
+    <col width="16" customWidth="1" min="39" max="39"/>
+    <col width="16" customWidth="1" min="40" max="40"/>
+    <col width="16" customWidth="1" min="41" max="41"/>
+    <col width="16" customWidth="1" min="42" max="42"/>
+    <col width="16" customWidth="1" min="43" max="43"/>
+    <col width="16" customWidth="1" min="44" max="44"/>
+    <col width="16" customWidth="1" min="45" max="45"/>
+    <col width="16" customWidth="1" min="46" max="46"/>
+    <col width="16" customWidth="1" min="47" max="47"/>
+    <col width="16" customWidth="1" min="48" max="48"/>
+    <col width="16" customWidth="1" min="49" max="49"/>
+    <col width="16" customWidth="1" min="50" max="50"/>
+    <col width="16" customWidth="1" min="51" max="51"/>
+    <col width="16" customWidth="1" min="52" max="52"/>
+    <col width="16" customWidth="1" min="53" max="53"/>
+    <col width="16" customWidth="1" min="54" max="54"/>
+    <col width="16" customWidth="1" min="55" max="55"/>
+    <col width="16" customWidth="1" min="56" max="56"/>
+    <col width="16" customWidth="1" min="57" max="57"/>
+    <col width="16" customWidth="1" min="58" max="58"/>
+    <col width="16" customWidth="1" min="59" max="59"/>
+    <col width="16" customWidth="1" min="60" max="60"/>
+    <col width="16" customWidth="1" min="61" max="61"/>
+    <col width="16" customWidth="1" min="62" max="62"/>
+    <col width="16" customWidth="1" min="63" max="63"/>
+    <col width="16" customWidth="1" min="64" max="64"/>
+    <col width="16" customWidth="1" min="65" max="65"/>
+    <col width="16" customWidth="1" min="66" max="66"/>
+    <col width="16" customWidth="1" min="67" max="67"/>
+    <col width="16" customWidth="1" min="68" max="68"/>
+    <col width="16" customWidth="1" min="69" max="69"/>
+    <col width="16" customWidth="1" min="70" max="70"/>
+    <col width="16" customWidth="1" min="71" max="71"/>
+    <col width="16" customWidth="1" min="72" max="72"/>
+    <col width="16" customWidth="1" min="73" max="73"/>
+    <col width="16" customWidth="1" min="74" max="74"/>
+    <col width="16" customWidth="1" min="75" max="75"/>
+    <col width="16" customWidth="1" min="76" max="76"/>
+    <col width="16" customWidth="1" min="77" max="77"/>
+    <col width="16" customWidth="1" min="78" max="78"/>
+    <col width="16" customWidth="1" min="79" max="79"/>
+    <col width="16" customWidth="1" min="80" max="80"/>
+    <col width="16" customWidth="1" min="81" max="81"/>
+    <col width="16" customWidth="1" min="82" max="82"/>
+    <col width="16" customWidth="1" min="83" max="83"/>
+    <col width="16" customWidth="1" min="84" max="84"/>
+    <col width="16" customWidth="1" min="85" max="85"/>
+    <col width="16" customWidth="1" min="86" max="86"/>
+    <col width="16" customWidth="1" min="87" max="87"/>
+    <col width="16" customWidth="1" min="88" max="88"/>
+    <col width="16" customWidth="1" min="89" max="89"/>
+    <col width="16" customWidth="1" min="90" max="90"/>
+    <col width="16" customWidth="1" min="91" max="91"/>
+    <col width="16" customWidth="1" min="92" max="92"/>
+    <col width="16" customWidth="1" min="93" max="93"/>
+    <col width="16" customWidth="1" min="94" max="94"/>
+    <col width="16" customWidth="1" min="95" max="95"/>
+    <col width="16" customWidth="1" min="96" max="96"/>
+    <col width="16" customWidth="1" min="97" max="97"/>
+    <col width="16" customWidth="1" min="98" max="98"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>AgentCode</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>AgentName</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>AppointDate</t>
+          <t>REGION_CODE</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>WorkModel</t>
+          <t>REGION_NAME</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>TerminateDate</t>
+          <t>ZONE_CODE</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>ZONE_NAME</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>BRANCH_CODE</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>BRANCH_NAME</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>SH_CODE</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>SH_NAME</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>SD_CODE</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>SD_NAME</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>INDIRECT 2_NAME</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>INDIRECT 2_NAME</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>INDIRECT 1_CODE</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>INDIRECT 1_NAME</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT_MANAGER_CODE</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT_MANAGER_NAME</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>LEADER</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>EXT_REF</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>AGENT_CODE</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>FULL_NAME</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>GENDER</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>TITLE (Code)</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>AGENT_STATUS</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>DOB</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>NATIONAL_ID</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>ID_ISSUE_DATE</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>ID_ISSUED_BY</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>ID_EXPIRATION_DATE</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>OLD_ID_NO</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>PLACE_OF_BIRTH</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>NATIONALITY</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>MARITAL_STATUS</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
+        <is>
+          <t>TAX_CODE</t>
+        </is>
+      </c>
+      <c r="AJ1" s="2" t="inlineStr">
+        <is>
+          <t>INCOME_RANGE</t>
+        </is>
+      </c>
+      <c r="AK1" s="2" t="inlineStr">
+        <is>
+          <t>EDUCATION</t>
+        </is>
+      </c>
+      <c r="AL1" s="2" t="inlineStr">
+        <is>
+          <t>PUBLIC_SECTOR</t>
+        </is>
+      </c>
+      <c r="AM1" s="2" t="inlineStr">
+        <is>
+          <t>OCCUPATION</t>
+        </is>
+      </c>
+      <c r="AN1" s="2" t="inlineStr">
+        <is>
+          <t>EXPERIENCE (Year)</t>
+        </is>
+      </c>
+      <c r="AO1" s="2" t="inlineStr">
+        <is>
+          <t>PERM_PROVINCE</t>
+        </is>
+      </c>
+      <c r="AP1" s="2" t="inlineStr">
+        <is>
+          <t>PERM_WARD</t>
+        </is>
+      </c>
+      <c r="AQ1" s="2" t="inlineStr">
+        <is>
+          <t>PERM_STREET</t>
+        </is>
+      </c>
+      <c r="AR1" s="2" t="inlineStr">
+        <is>
+          <t>CONTACT_PROVINCE</t>
+        </is>
+      </c>
+      <c r="AS1" s="2" t="inlineStr">
+        <is>
+          <t>CONTACT_WARD</t>
+        </is>
+      </c>
+      <c r="AT1" s="2" t="inlineStr">
+        <is>
+          <t>CONTACT_STREET</t>
+        </is>
+      </c>
+      <c r="AU1" s="2" t="inlineStr">
+        <is>
+          <t>MOBILE</t>
+        </is>
+      </c>
+      <c r="AV1" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAL_EMAIL</t>
+        </is>
+      </c>
+      <c r="AW1" s="2" t="inlineStr">
+        <is>
+          <t>COMPANY_EMAIL</t>
+        </is>
+      </c>
+      <c r="AX1" s="2" t="inlineStr">
+        <is>
+          <t>CHANNEL</t>
+        </is>
+      </c>
+      <c r="AY1" s="2" t="inlineStr">
+        <is>
+          <t>AGENCY_TYPE</t>
+        </is>
+      </c>
+      <c r="AZ1" s="2" t="inlineStr">
+        <is>
+          <t>FIRST_RECRUITER_CODE</t>
+        </is>
+      </c>
+      <c r="BA1" s="2" t="inlineStr">
+        <is>
+          <t>REFERRER_CODE</t>
+        </is>
+      </c>
+      <c r="BB1" s="2" t="inlineStr">
+        <is>
+          <t>APPOINTMENT_DATE</t>
+        </is>
+      </c>
+      <c r="BC1" s="2" t="inlineStr">
+        <is>
+          <t>TERMINATION_DATE</t>
+        </is>
+      </c>
+      <c r="BD1" s="2" t="inlineStr">
+        <is>
+          <t>FIRST APPOINTMENT_DATE</t>
+        </is>
+      </c>
+      <c r="BE1" s="2" t="inlineStr">
+        <is>
+          <t>PROMOTION_DATE</t>
+        </is>
+      </c>
+      <c r="BF1" s="2" t="inlineStr">
+        <is>
+          <t>DEMOTION_DATE</t>
+        </is>
+      </c>
+      <c r="BG1" s="2" t="inlineStr">
+        <is>
+          <t>BANK_ACCOUNT_HOLDER</t>
+        </is>
+      </c>
+      <c r="BH1" s="2" t="inlineStr">
+        <is>
+          <t>BANK_ACCOUNT_NO</t>
+        </is>
+      </c>
+      <c r="BI1" s="2" t="inlineStr">
+        <is>
+          <t>BANK_CODE</t>
+        </is>
+      </c>
+      <c r="BJ1" s="2" t="inlineStr">
+        <is>
+          <t>BANK_BRANCH</t>
+        </is>
+      </c>
+      <c r="BK1" s="2" t="inlineStr">
+        <is>
+          <t>BANK_BRANCH CODE (Payment)</t>
+        </is>
+      </c>
+      <c r="BL1" s="2" t="inlineStr">
+        <is>
+          <t>MOF_CERT_NO</t>
+        </is>
+      </c>
+      <c r="BM1" s="2" t="inlineStr">
+        <is>
+          <t>MOF_CERT_ISSUE_DATE</t>
+        </is>
+      </c>
+      <c r="BN1" s="2" t="inlineStr">
+        <is>
+          <t>MOF_EXAM_PASS_DATE</t>
+        </is>
+      </c>
+      <c r="BO1" s="2" t="inlineStr">
+        <is>
+          <t>AVICAD_STATUS</t>
+        </is>
+      </c>
+      <c r="BP1" s="2" t="inlineStr">
+        <is>
+          <t>AVICAD_DESC</t>
+        </is>
+      </c>
+      <c r="BQ1" s="2" t="inlineStr">
+        <is>
+          <t>AVICAD_CHECKED_AT</t>
+        </is>
+      </c>
+      <c r="BR1" s="2" t="inlineStr">
+        <is>
+          <t>CONTRACT_NO Agent</t>
+        </is>
+      </c>
+      <c r="BS1" s="2" t="inlineStr">
+        <is>
+          <t>CONTRACT_TYPE</t>
+        </is>
+      </c>
+      <c r="BT1" s="2" t="inlineStr">
+        <is>
+          <t>CONTRACT_NO Leader</t>
+        </is>
+      </c>
+      <c r="BU1" s="2" t="inlineStr">
+        <is>
+          <t>CONTRACT_TYPE</t>
+        </is>
+      </c>
+      <c r="BV1" s="2" t="inlineStr">
+        <is>
+          <t>ESIGN_ENVELOPE_ID (DOCUMENT ID)</t>
+        </is>
+      </c>
+      <c r="BW1" s="2" t="inlineStr">
+        <is>
+          <t>CONTRACT_SENT_DATE</t>
+        </is>
+      </c>
+      <c r="BX1" s="2" t="inlineStr">
+        <is>
+          <t>CONTRACT_SIGNED_DATE</t>
+        </is>
+      </c>
+      <c r="BY1" s="2" t="inlineStr">
+        <is>
+          <t>SIGN_AUTH_METHOD</t>
+        </is>
+      </c>
+      <c r="BZ1" s="2" t="inlineStr">
+        <is>
+          <t>SIGN_STATUS</t>
+        </is>
+      </c>
+      <c r="CA1" s="2" t="inlineStr">
+        <is>
+          <t>CONTRACT_FILE_NAME</t>
+        </is>
+      </c>
+      <c r="CB1" s="2" t="inlineStr">
+        <is>
+          <t>CONTRACT_DMS_REF</t>
+        </is>
+      </c>
+      <c r="CC1" s="2" t="inlineStr">
+        <is>
+          <t>PROGRAM_CODES</t>
+        </is>
+      </c>
+      <c r="CD1" s="2" t="inlineStr">
+        <is>
+          <t>COMMIT_1</t>
+        </is>
+      </c>
+      <c r="CE1" s="2" t="inlineStr">
+        <is>
+          <t>COMMIT_2</t>
+        </is>
+      </c>
+      <c r="CF1" s="2" t="inlineStr">
+        <is>
+          <t>COMMIT_3</t>
+        </is>
+      </c>
+      <c r="CG1" s="2" t="inlineStr">
+        <is>
+          <t>COMMIT_4</t>
+        </is>
+      </c>
+      <c r="CH1" s="2" t="inlineStr">
+        <is>
+          <t>CONSENT_NOTIFY_OPS</t>
+        </is>
+      </c>
+      <c r="CI1" s="2" t="inlineStr">
+        <is>
+          <t>CONSENT_NOTIFY_PROMO</t>
+        </is>
+      </c>
+      <c r="CJ1" s="2" t="inlineStr">
+        <is>
+          <t>PDPD_1_BASIC</t>
+        </is>
+      </c>
+      <c r="CK1" s="2" t="inlineStr">
+        <is>
+          <t>PDPD_2_SENSITIVE</t>
+        </is>
+      </c>
+      <c r="CL1" s="2" t="inlineStr">
+        <is>
+          <t>PDPD_3_SHARE</t>
+        </is>
+      </c>
+      <c r="CM1" s="2" t="inlineStr">
+        <is>
+          <t>CONSENT_DATE</t>
+        </is>
+      </c>
+      <c r="CN1" s="2" t="inlineStr">
+        <is>
+          <t>CONSENT_METHOD</t>
+        </is>
+      </c>
+      <c r="CO1" s="2" t="inlineStr">
+        <is>
+          <t>ONBOARD_COURSE_CODE</t>
+        </is>
+      </c>
+      <c r="CP1" s="2" t="inlineStr">
+        <is>
+          <t>ONBOARD_COURSE_DATE</t>
+        </is>
+      </c>
+      <c r="CQ1" s="2" t="inlineStr">
+        <is>
+          <t>TRAINING_COMPLETED</t>
+        </is>
+      </c>
+      <c r="CR1" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_AUTH_CODES</t>
+        </is>
+      </c>
+      <c r="CS1" s="2" t="inlineStr">
+        <is>
+          <t>DOC_RECEIVED</t>
+        </is>
+      </c>
+      <c r="CT1" s="2" t="inlineStr">
+        <is>
+          <t>DOC_DMS_REF</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>LP001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>LP A (ví dụ văn bản)</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="n"/>
+      <c r="AB2" s="4" t="n"/>
+      <c r="AD2" s="4" t="n"/>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+      <c r="BB2" s="4" t="n">
         <v>46083</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="BC2" s="4" t="n"/>
+      <c r="BD2" s="4" t="n"/>
+      <c r="BE2" s="4" t="n"/>
+      <c r="BF2" s="4" t="n"/>
+      <c r="BM2" s="4" t="n"/>
+      <c r="BN2" s="4" t="n"/>
+      <c r="BQ2" s="4" t="n"/>
+      <c r="BW2" s="4" t="n"/>
+      <c r="BX2" s="4" t="n"/>
+      <c r="CM2" s="4" t="n"/>
+      <c r="CP2" s="4" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>LP002</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn B</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z3" s="4" t="n"/>
+      <c r="AB3" s="4" t="n"/>
+      <c r="AD3" s="4" t="n"/>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="BB3" s="4" t="n">
+        <v>45810</v>
+      </c>
+      <c r="BC3" s="4" t="n"/>
+      <c r="BD3" s="4" t="n"/>
+      <c r="BE3" s="4" t="n"/>
+      <c r="BF3" s="4" t="n"/>
+      <c r="BM3" s="4" t="n"/>
+      <c r="BN3" s="4" t="n"/>
+      <c r="BQ3" s="4" t="n"/>
+      <c r="BW3" s="4" t="n"/>
+      <c r="BX3" s="4" t="n"/>
+      <c r="CM3" s="4" t="n"/>
+      <c r="CP3" s="4" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>LP003</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Trần Thị C</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LP002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Nguyễn Văn B</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>45810</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z4" s="4" t="n"/>
+      <c r="AB4" s="4" t="n"/>
+      <c r="AD4" s="4" t="n"/>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="BB4" s="4" t="n">
+        <v>46027</v>
+      </c>
+      <c r="BC4" s="4" t="n"/>
+      <c r="BD4" s="4" t="n"/>
+      <c r="BE4" s="4" t="n"/>
+      <c r="BF4" s="4" t="n"/>
+      <c r="BM4" s="4" t="n"/>
+      <c r="BN4" s="4" t="n"/>
+      <c r="BQ4" s="4" t="n"/>
+      <c r="BW4" s="4" t="n"/>
+      <c r="BX4" s="4" t="n"/>
+      <c r="CM4" s="4" t="n"/>
+      <c r="CP4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>LP004</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Lê Văn D</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>LP003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Trần Thị C</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>46027</v>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z5" s="4" t="n"/>
+      <c r="AB5" s="4" t="n"/>
+      <c r="AD5" s="4" t="n"/>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="BB5" s="4" t="n">
+        <v>45901</v>
+      </c>
+      <c r="BC5" s="4" t="n"/>
+      <c r="BD5" s="4" t="n"/>
+      <c r="BE5" s="4" t="n"/>
+      <c r="BF5" s="4" t="n"/>
+      <c r="BM5" s="4" t="n"/>
+      <c r="BN5" s="4" t="n"/>
+      <c r="BQ5" s="4" t="n"/>
+      <c r="BW5" s="4" t="n"/>
+      <c r="BX5" s="4" t="n"/>
+      <c r="CM5" s="4" t="n"/>
+      <c r="CP5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>LP005</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Phạm Thị E</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>LP004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Lê Văn D</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>45901</v>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z6" s="4" t="n"/>
+      <c r="AB6" s="4" t="n"/>
+      <c r="AD6" s="4" t="n"/>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="BB6" s="4" t="n">
+        <v>46055</v>
+      </c>
+      <c r="BC6" s="4" t="n"/>
+      <c r="BD6" s="4" t="n"/>
+      <c r="BE6" s="4" t="n"/>
+      <c r="BF6" s="4" t="n"/>
+      <c r="BM6" s="4" t="n"/>
+      <c r="BN6" s="4" t="n"/>
+      <c r="BQ6" s="4" t="n"/>
+      <c r="BW6" s="4" t="n"/>
+      <c r="BX6" s="4" t="n"/>
+      <c r="CM6" s="4" t="n"/>
+      <c r="CP6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>LP006</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Hoàng Văn F</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>LP005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Phạm Thị E</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>46055</v>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z7" s="4" t="n"/>
+      <c r="AB7" s="4" t="n"/>
+      <c r="AD7" s="4" t="n"/>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="BB7" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="BC7" s="4" t="n"/>
+      <c r="BD7" s="4" t="n"/>
+      <c r="BE7" s="4" t="n"/>
+      <c r="BF7" s="4" t="n"/>
+      <c r="BM7" s="4" t="n"/>
+      <c r="BN7" s="4" t="n"/>
+      <c r="BQ7" s="4" t="n"/>
+      <c r="BW7" s="4" t="n"/>
+      <c r="BX7" s="4" t="n"/>
+      <c r="CM7" s="4" t="n"/>
+      <c r="CP7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>LP007</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Vũ Thị G</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>LP006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Hoàng Văn F</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="n">
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z8" s="4" t="n"/>
+      <c r="AB8" s="4" t="n"/>
+      <c r="AD8" s="4" t="n"/>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+      <c r="BB8" s="4" t="n">
         <v>46307</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="BC8" s="4" t="n"/>
+      <c r="BD8" s="4" t="n"/>
+      <c r="BE8" s="4" t="n"/>
+      <c r="BF8" s="4" t="n"/>
+      <c r="BM8" s="4" t="n"/>
+      <c r="BN8" s="4" t="n"/>
+      <c r="BQ8" s="4" t="n"/>
+      <c r="BW8" s="4" t="n"/>
+      <c r="BX8" s="4" t="n"/>
+      <c r="CM8" s="4" t="n"/>
+      <c r="CP8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>LP008</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Đặng Văn H</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z9" s="4" t="n"/>
+      <c r="AB9" s="4" t="n"/>
+      <c r="AD9" s="4" t="n"/>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="BB9" s="4" t="n">
+        <v>45964</v>
+      </c>
+      <c r="BC9" s="4" t="n"/>
+      <c r="BD9" s="4" t="n"/>
+      <c r="BE9" s="4" t="n"/>
+      <c r="BF9" s="4" t="n"/>
+      <c r="BM9" s="4" t="n"/>
+      <c r="BN9" s="4" t="n"/>
+      <c r="BQ9" s="4" t="n"/>
+      <c r="BW9" s="4" t="n"/>
+      <c r="BX9" s="4" t="n"/>
+      <c r="CM9" s="4" t="n"/>
+      <c r="CP9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>LP009</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Bùi Thị I</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>LP</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z10" s="4" t="n"/>
+      <c r="AB10" s="4" t="n"/>
+      <c r="AD10" s="4" t="n"/>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="BB10" s="4" t="n">
+        <v>46113</v>
+      </c>
+      <c r="BC10" s="4" t="n"/>
+      <c r="BD10" s="4" t="n"/>
+      <c r="BE10" s="4" t="n"/>
+      <c r="BF10" s="4" t="n"/>
+      <c r="BM10" s="4" t="n"/>
+      <c r="BN10" s="4" t="n"/>
+      <c r="BQ10" s="4" t="n"/>
+      <c r="BW10" s="4" t="n"/>
+      <c r="BX10" s="4" t="n"/>
+      <c r="CM10" s="4" t="n"/>
+      <c r="CP10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>LP010</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Đỗ Văn K</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>LP007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Vũ Thị G</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>46307</v>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z11" s="4" t="n"/>
+      <c r="AB11" s="4" t="n"/>
+      <c r="AD11" s="4" t="n"/>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>LP</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>LP008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Đặng Văn H</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>45964</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>PT</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>LP</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>LP009</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Bùi Thị I</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>46113</v>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="BB11" s="4" t="n">
+        <v>45870</v>
+      </c>
+      <c r="BC11" s="4" t="n"/>
+      <c r="BD11" s="4" t="n"/>
+      <c r="BE11" s="4" t="n"/>
+      <c r="BF11" s="4" t="n"/>
+      <c r="BM11" s="4" t="n"/>
+      <c r="BN11" s="4" t="n"/>
+      <c r="BQ11" s="4" t="n"/>
+      <c r="BW11" s="4" t="n"/>
+      <c r="BX11" s="4" t="n"/>
+      <c r="CM11" s="4" t="n"/>
+      <c r="CP11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>202610</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>PM001</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Ngô Thị M</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Z12" s="4" t="n"/>
+      <c r="AB12" s="4" t="n"/>
+      <c r="AD12" s="4" t="n"/>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>LP</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LP010</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Đỗ Văn K</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>45870</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>LP</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>PM001</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Ngô Thị M</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="n">
+      <c r="BB12" s="4" t="n">
         <v>46083</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>PM</t>
-        </is>
-      </c>
+      <c r="BC12" s="4" t="n"/>
+      <c r="BD12" s="4" t="n"/>
+      <c r="BE12" s="4" t="n"/>
+      <c r="BF12" s="4" t="n"/>
+      <c r="BM12" s="4" t="n"/>
+      <c r="BN12" s="4" t="n"/>
+      <c r="BQ12" s="4" t="n"/>
+      <c r="BW12" s="4" t="n"/>
+      <c r="BX12" s="4" t="n"/>
+      <c r="CM12" s="4" t="n"/>
+      <c r="CP12" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -966,7 +1878,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="4" t="n">
         <v>46267</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -976,7 +1888,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="4" t="n">
         <v>46388</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -1070,7 +1982,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1108,7 +2020,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1149,7 +2061,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1190,7 +2102,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1231,7 +2143,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1269,7 +2181,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1307,7 +2219,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1345,7 +2257,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1386,7 +2298,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1424,7 +2336,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>
@@ -1465,7 +2377,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>202610</t>
         </is>

</xml_diff>